<commit_message>
feat: upgrade telegram layout, resolve proxy timeouts, and add manual captcha solver
</commit_message>
<xml_diff>
--- a/running shoes.xlsx
+++ b/running shoes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Desktop" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Desktop" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Mobile" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,257 +414,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="B1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Keyword</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>URLs</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Type</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>running shoes</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.nike.com/w/running-shoes-37v7jzy7ok</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>10-01-2024</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Competitor</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>running shoes</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.adidas.com/us/women-running-shoes</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>10-01-2024</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>My Site</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>running shoes</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>9</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.hoka.com/en/us/</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>10-01-2024</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Competitor</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>running shoes</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>13</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.adidas.com/us/running-shoes</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>10-01-2024</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>My Site</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>running shoes</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>23</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>https://www.reebok.com/c/200000012/men-running-shoes</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>10-01-2024</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Competitor</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>running shoes</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>42</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>https://www.nike.com/running</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>10-01-2024</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Competitor</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>running shoes</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>66</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>https://www.hoka.com/en/us/mens-road/</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>10-01-2024</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Competitor</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>running shoes</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>90</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>https://www.reebok.com/c/100000014/women-running-shoes</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>10-01-2024</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Competitor</t>
         </is>
       </c>
     </row>
@@ -691,145 +455,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="B1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Keyword</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>URLs</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Type</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>running shoes</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>https://www.nike.com/w/running-shoes-37v7jzy7ok</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>10-01-2024</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Competitor</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>running shoes</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>https://www.adidas.com/us/women-running-shoes</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>10-01-2024</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>My Site</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>running shoes</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>8</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>https://www.hoka.com/en/us/</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>10-01-2024</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Competitor</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>running shoes</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>23</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>https://www.reebok.com/c/200000012/men-running-shoes</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>10-01-2024</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Competitor</t>
         </is>
       </c>
     </row>

</xml_diff>